<commit_message>
modificaciones en varios directorios
</commit_message>
<xml_diff>
--- a/app/files/mimasoft_files/client_1/project_1/form_4/LAG_EC1Energía-Electricidad_plantilla.xlsx
+++ b/app/files/mimasoft_files/client_1/project_1/form_4/LAG_EC1Energía-Electricidad_plantilla.xlsx
@@ -562,28 +562,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="0" t="s">
         <v>7</v>
       </c>
     </row>
@@ -591,25 +591,25 @@
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="0" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="0">
         <v>2023</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="0" t="s">
         <v>14</v>
       </c>
     </row>
@@ -656,42 +656,42 @@
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="E1">
+      <c r="E1" s="0">
         <v>2023</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="D2" t="s">
+      <c r="D2" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="0">
         <v>2024</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="D3" t="s">
+      <c r="D3" s="0" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="D4" t="s">
+      <c r="D4" s="0" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="D5" t="s">
+      <c r="D5" s="0" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>